<commit_message>
Foreign rrp formatting fix
</commit_message>
<xml_diff>
--- a/backend/public/templates/template_file.xlsx
+++ b/backend/public/templates/template_file.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Request Template" sheetId="1" state="visible" r:id="rId3"/>
@@ -2419,9 +2419,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1645560</xdr:colOff>
+      <xdr:colOff>1645200</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>169200</xdr:rowOff>
+      <xdr:rowOff>168840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2435,7 +2435,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1856880" cy="664560"/>
+          <a:ext cx="1856520" cy="664200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2462,9 +2462,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1578960</xdr:colOff>
+      <xdr:colOff>1578600</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>157320</xdr:rowOff>
+      <xdr:rowOff>156960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2478,7 +2478,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1860840" cy="664560"/>
+          <a:ext cx="1860480" cy="664200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2505,9 +2505,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>967680</xdr:colOff>
+      <xdr:colOff>967320</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>102600</xdr:rowOff>
+      <xdr:rowOff>102240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2521,7 +2521,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1360080" cy="483480"/>
+          <a:ext cx="1359720" cy="483120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2548,9 +2548,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1388160</xdr:colOff>
+      <xdr:colOff>1387800</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>35640</xdr:rowOff>
+      <xdr:rowOff>35280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2564,7 +2564,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1951920" cy="506160"/>
+          <a:ext cx="1951560" cy="505800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Foreign rrp formatting fix (#36)
</commit_message>
<xml_diff>
--- a/backend/public/templates/template_file.xlsx
+++ b/backend/public/templates/template_file.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Request Template" sheetId="1" state="visible" r:id="rId3"/>
@@ -2419,9 +2419,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1645560</xdr:colOff>
+      <xdr:colOff>1645200</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>169200</xdr:rowOff>
+      <xdr:rowOff>168840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2435,7 +2435,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1856880" cy="664560"/>
+          <a:ext cx="1856520" cy="664200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2462,9 +2462,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1578960</xdr:colOff>
+      <xdr:colOff>1578600</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>157320</xdr:rowOff>
+      <xdr:rowOff>156960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2478,7 +2478,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1860840" cy="664560"/>
+          <a:ext cx="1860480" cy="664200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2505,9 +2505,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>967680</xdr:colOff>
+      <xdr:colOff>967320</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>102600</xdr:rowOff>
+      <xdr:rowOff>102240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2521,7 +2521,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1360080" cy="483480"/>
+          <a:ext cx="1359720" cy="483120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2548,9 +2548,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1388160</xdr:colOff>
+      <xdr:colOff>1387800</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>35640</xdr:rowOff>
+      <xdr:rowOff>35280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2564,7 +2564,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1951920" cy="506160"/>
+          <a:ext cx="1951560" cy="505800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>